<commit_message>
fix(audit): resolve all 24 critical/high/medium/low audit findings (v65.0)
</commit_message>
<xml_diff>
--- a/data/blank_template_smart_money.xlsx
+++ b/data/blank_template_smart_money.xlsx
@@ -610,7 +610,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
@@ -685,7 +685,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -760,7 +760,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">

</xml_diff>